<commit_message>
Refactor subscription handling: rename renewalDate to endDate, add endDateNoSkip; update related logic and UI components
- Introduced ScenarioCard component for better code organization in TestingPage.
- Updated CustomerNameWithNote and CustomerOverlayTrigger components to improve note display.
- Modified CustomerOverlay and SchedulePanel components to accommodate new subscription end date logic.
- Adjusted utility functions to work with endDate instead of renewalDate.
- Migrated selections to use subscriptionId instead of customerId, ensuring data integrity.
- Updated seed and testing scripts to reflect changes in subscription structure.
</commit_message>
<xml_diff>
--- a/data/test/menu.xlsx
+++ b/data/test/menu.xlsx
@@ -430,10 +430,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-W19-1-1</v>
+        <v>2026-W20-1-1</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -456,10 +456,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-W19-1-2</v>
+        <v>2026-W20-1-2</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -482,10 +482,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-W19-2-1</v>
+        <v>2026-W20-2-1</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -508,10 +508,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-W19-2-2</v>
+        <v>2026-W20-2-2</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -534,10 +534,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-W19-3-1</v>
+        <v>2026-W20-3-1</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C6">
         <v>3</v>
@@ -560,10 +560,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-W19-3-2</v>
+        <v>2026-W20-3-2</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C7">
         <v>3</v>
@@ -586,10 +586,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-W19-4-1</v>
+        <v>2026-W20-4-1</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C8">
         <v>4</v>
@@ -612,10 +612,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-W19-4-2</v>
+        <v>2026-W20-4-2</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C9">
         <v>4</v>
@@ -638,10 +638,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-W19-5-1</v>
+        <v>2026-W20-5-1</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C10">
         <v>5</v>
@@ -664,10 +664,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-W19-5-2</v>
+        <v>2026-W20-5-2</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-W19</v>
+        <v>2026-W20</v>
       </c>
       <c r="C11">
         <v>5</v>
@@ -690,10 +690,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-W20-1-1</v>
+        <v>2026-W21-1-1</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -716,10 +716,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-W20-1-2</v>
+        <v>2026-W21-1-2</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -742,10 +742,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-W20-2-1</v>
+        <v>2026-W21-2-1</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -768,10 +768,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-W20-2-2</v>
+        <v>2026-W21-2-2</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -794,10 +794,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-W20-3-1</v>
+        <v>2026-W21-3-1</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C16">
         <v>3</v>
@@ -820,10 +820,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-W20-3-2</v>
+        <v>2026-W21-3-2</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C17">
         <v>3</v>
@@ -846,10 +846,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-W20-4-1</v>
+        <v>2026-W21-4-1</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C18">
         <v>4</v>
@@ -872,10 +872,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-W20-4-2</v>
+        <v>2026-W21-4-2</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C19">
         <v>4</v>
@@ -898,10 +898,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-W20-5-1</v>
+        <v>2026-W21-5-1</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C20">
         <v>5</v>
@@ -924,10 +924,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-W20-5-2</v>
+        <v>2026-W21-5-2</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-W20</v>
+        <v>2026-W21</v>
       </c>
       <c r="C21">
         <v>5</v>

</xml_diff>